<commit_message>
1. removed "CTD_" prefixes from table names and column names, 2. removed CTD_INSTRUMENT_CODES table creation code and references, 3. folded instrument codes into the ENVIRONMENTAL table (previously CTD_DATA), 4. changed the VAR_NAME column to NAME, in keeping with our naming definitions in METADATA_COLUMN table, 5. updated the create_ctd_view.sql table to match the new column names and table names, 6. updated fields in ctd_lookup_table_data.xlsx to match new column names.
</commit_message>
<xml_diff>
--- a/code/ctd_data/ctd_lookup_table_data.xlsx
+++ b/code/ctd_data/ctd_lookup_table_data.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zack.oyafuso\Work\GitHub\gap_products\code\ctd_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Projects\gap_products_general\gap_products\code\ctd_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73C13465-E5D9-4C29-98FA-9661D2E60382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{257A6C10-C573-41A2-8D71-44026AE3E45F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="16440" windowHeight="28320" activeTab="2" xr2:uid="{60C4621A-9269-41C1-A8ED-C4F6743386D3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{60C4621A-9269-41C1-A8ED-C4F6743386D3}"/>
   </bookViews>
   <sheets>
-    <sheet name="CTD_DIRECTION_CODES" sheetId="1" r:id="rId1"/>
-    <sheet name="CTD_INSTRUMENT_CODES" sheetId="2" r:id="rId2"/>
-    <sheet name="CTD_VARIABLE_CODES" sheetId="3" r:id="rId3"/>
+    <sheet name="DIRECTION_CODES" sheetId="1" r:id="rId1"/>
+    <sheet name="INSTRUMENT_CODES" sheetId="2" r:id="rId2"/>
+    <sheet name="VARIABLE_CODES" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,9 +31,6 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -77,9 +74,6 @@
     <t>VARIABLE</t>
   </si>
   <si>
-    <t>VAR_NAME</t>
-  </si>
-  <si>
     <t>UNITS</t>
   </si>
   <si>
@@ -180,6 +174,9 @@
   </si>
   <si>
     <t>Conductivity in Sieverts per meter</t>
+  </si>
+  <si>
+    <t>NAME</t>
   </si>
 </sst>
 </file>
@@ -532,13 +529,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84231558-C7AB-468B-A656-8E5D5EFF8522}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -546,7 +543,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>-1</v>
       </c>
@@ -554,7 +551,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>0</v>
       </c>
@@ -562,7 +559,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>1</v>
       </c>
@@ -578,13 +575,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14E53FDA-BFF1-4D9A-887E-2320C73981AD}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="57.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="57.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>10</v>
       </c>
@@ -592,7 +589,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -600,7 +597,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -608,7 +605,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -616,7 +613,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -624,7 +621,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -640,188 +637,188 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C49F0285-8574-4C4B-A78A-F3EFD693CA3C}">
   <dimension ref="A1:D13"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="58.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="58.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>11</v>
       </c>
       <c r="B1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1" t="s">
         <v>12</v>
-      </c>
-      <c r="C1" t="s">
-        <v>13</v>
       </c>
       <c r="D1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" t="s">
         <v>35</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>36</v>
       </c>
-      <c r="D3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" t="s">
         <v>38</v>
       </c>
-      <c r="C5" t="s">
-        <v>39</v>
-      </c>
       <c r="D5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" t="s">
         <v>40</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>41</v>
       </c>
-      <c r="D7" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D8" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D9" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D10" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" t="s">
         <v>44</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>45</v>
-      </c>
-      <c r="D13" t="s">
-        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>